<commit_message>
Restore explicit Extreme prompts and expand that style
Add back the 20 explicit/taboo Extreme prompts dropped in the earlier
mature rewrite (they were the intended tone for the Extreme tier), reworded
to match the deck's voice and the 1-3 drink scale, and build out ~27 more
in the same explicit confessional/dare vein across three new sections:
Drink If (Explicit Acts), Drink If (Taboo & Wild), Drink If (Paid &
Provocative) and Explicit Dares (Hands & Simulation).

Extreme 192->239; deck now 486 prompts. Regenerated the CSV and the
two-tab workbook (the restored prompts now show as 'Re-added').

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AREzGtAYjLvz5Af3E4CcDP
</commit_message>
<xml_diff>
--- a/docs/afterhours-prompts.xlsx
+++ b/docs/afterhours-prompts.xlsx
@@ -9697,6 +9697,1040 @@
         </is>
       </c>
     </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">492</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever swallowed; if you never have, take 2 instead.</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">493</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever let someone finish on your face.</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">494</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever been double-penetrated.</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">495</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever given or received a golden shower.</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">496</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever been fisted, or done the fisting.</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">497</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had sex on your period.</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">498</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever done anal without lube; respect.</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">499</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever used a butt plug in the bedroom.</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">500</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever been spit on in bed and liked it.</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">501</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever squirted, or made someone else.</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">502</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had a hand around your throat and asked for more.</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">503</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever finished more than once in a single session.</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">504</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever deep-throated, dare or otherwise.</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">505</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever tasted yourself.</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">506</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever rimmed someone, or been rimmed.</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">507</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever pegged someone, or been pegged.</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">508</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever left nail marks down someone's back.</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">509</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever come so hard you saw stars.</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Explicit Acts)</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">510</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had sex in a church, temple, or anywhere holy.</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">511</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever hooked up at a funeral or a wedding.</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">512</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever hooked up with a family member's friend.</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">513</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever slept with someone 15+ years older or younger than you.</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">514</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever slept with a friend's ex and never confessed.</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">515</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had sex at your workplace after hours.</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">516</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever hooked up with someone twice your age.</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">517</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever been the other person in an affair.</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">518</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever hooked up with two people in the same night.</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">519</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever hooked up with someone you wouldn't dare name out loud.</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">520</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had sex in your childhood bedroom as a grown adult.</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Taboo &amp; Wild)</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">521</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever been paid for anything sexual; strip a layer if yes.</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Paid &amp; Provocative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">522</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had a sugar daddy or sugar mommy; lose a layer if it's still active.</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Paid &amp; Provocative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">523</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever paid for sex; admit it or lose a layer.</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Paid &amp; Provocative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">524</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever made money from a photo of yourself.</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Paid &amp; Provocative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">525</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink if you've ever had a spicy subscription account, or paid for someone else's.</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Drink If (Paid &amp; Provocative)</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">526</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} slip a hand into your waistband for 10 seconds, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">527</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Slide a hand under {{randomOtherPlayer}}'s clothes and tease for 15 seconds, or drink 3.</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">528</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} undo your pants and slip a hand exactly where they like, or finish your drink.</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">529</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suck {{randomOtherPlayer}}'s toe like you actually mean it, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">530</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Guide {{randomOtherPlayer}}'s hand exactly where you'd want it and hold it there for 10 seconds, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">531</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} decide where your hands go for the next 20 seconds, or drink 3.</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">532</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulate going down on {{randomOtherPlayer}} for 10 seconds, fully clothed, or finish your drink.</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">533</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} grind against your thigh until the song changes, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t xml:space="preserve">534</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Whisper to {{randomOtherPlayer}} exactly how you'd finish them off, or drink 3.</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t xml:space="preserve">535</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Put two fingers in {{randomOtherPlayer}}'s mouth and let them show you what they'd do, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t xml:space="preserve">536</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kiss and bite your way down {{randomOtherPlayer}}'s stomach to their waistband, or finish your drink.</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">537</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Press against {{randomOtherPlayer}} from behind and set the pace for 15 seconds, or drink 3.</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">538</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} slide your underwear off using only their teeth, or take 3 drinks.</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Extreme</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Explicit Dares (Hands &amp; Simulation)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -11430,12 +12464,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14238,12 +15272,12 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14265,12 +15299,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14400,12 +15434,12 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14778,12 +15812,12 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14859,12 +15893,12 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14886,12 +15920,12 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14913,12 +15947,12 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14940,12 +15974,12 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14967,12 +16001,12 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -14994,12 +16028,12 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15021,12 +16055,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15237,12 +16271,12 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15372,12 +16406,12 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15399,12 +16433,12 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15588,12 +16622,12 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15642,12 +16676,12 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15669,12 +16703,12 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15696,12 +16730,12 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>
@@ -15723,12 +16757,12 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cut</t>
+          <t xml:space="preserve">Re-added</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Too graphic / taboo for the mature rewrite; no equivalent kept.</t>
+          <t xml:space="preserve">Dropped in the first rewrite, added back per request and reworded to match the deck voice.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recalibrate Mild and Medium tiers hornier for a late-night crowd
Per feedback that 'more mature' meant more adult/risque/sexier (drunk and
sexual), not tamer:

- Mild (82) rewritten as an openly suggestive warm-up: turn-ons, attraction
  and body talk, sexy this-or-that, flirty light dares and flirty drink-ifs.
  Still clothed with no explicit acts, so it stays the entry tier.
- Medium (165) rewritten overtly sexual and escalating toward the Extreme
  border: dirty confessions and questions, sexual-history drink-ifs,
  hands-on (clothed) dares, sexting/phone stunts, incentivized reveals and
  sexual drink commands.
- Extreme unchanged. Deck stays 486 prompts; drinks stay on the 1-3 scale.
  Regenerated CSV and the two-tab workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AREzGtAYjLvz5Af3E4CcDP
</commit_message>
<xml_diff>
--- a/docs/afterhours-prompts.xlsx
+++ b/docs/afterhours-prompts.xlsx
@@ -47,7 +47,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe yourself in three words your ex would strongly disagree with.</t>
+          <t xml:space="preserve">What's the first thing you notice on someone you're attracted to?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -57,7 +57,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -69,7 +69,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most flattering lie you tell people about yourself?</t>
+          <t xml:space="preserve">Describe your type in three words, then look around the room.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -79,7 +79,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -91,7 +91,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">If your life had a theme song that played when you walked in, what is it?</t>
+          <t xml:space="preserve">What's your go-to move when you want someone to notice you?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -101,7 +101,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -113,7 +113,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a strong opinion you'll defend with your whole chest and zero evidence?</t>
+          <t xml:space="preserve">Who was your most embarrassing crush, and what did they have going on?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -123,7 +123,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -135,7 +135,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal the pettiest reason you've ever disliked someone on sight.</t>
+          <t xml:space="preserve">What's the most attractive thing someone can wear?</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -145,7 +145,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -157,7 +157,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most unhinged thing in your search history you'll actually admit to?</t>
+          <t xml:space="preserve">Rate your own flirting skills out of 10, then let the group correct you.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -167,7 +167,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -179,7 +179,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">What compliment do you fish for the hardest?</t>
+          <t xml:space="preserve">What's a compliment that instantly makes you blush?</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -189,7 +189,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -201,7 +201,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal your most-used emoji and explain what that says about you.</t>
+          <t xml:space="preserve">What's the biggest green flag that makes you want someone immediately?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -211,7 +211,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -223,7 +223,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the last little white lie you told, and who you told it to.</t>
+          <t xml:space="preserve">Who in this room has the best trouble energy?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -233,7 +233,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -245,7 +245,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most embarrassing thing you've done to get someone's attention?</t>
+          <t xml:space="preserve">What's your most shameless way of getting someone's attention?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -255,7 +255,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -267,7 +267,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a secret talent you're quietly proud of but never bring up?</t>
+          <t xml:space="preserve">Describe your flirting style: smooth, chaotic, or hopeless?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -277,7 +277,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -289,7 +289,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell the group the last thing you Googled at 2am.</t>
+          <t xml:space="preserve">What's the fastest anyone has ever caught your eye?</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -299,7 +299,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -311,7 +311,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal the most embarrassing song in your most-played list.</t>
+          <t xml:space="preserve">Which emoji do you send when you're actually into someone?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -321,7 +321,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -333,7 +333,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the pettiest hill you've ever died on in an argument?</t>
+          <t xml:space="preserve">What instantly makes you lose interest in someone?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -343,7 +343,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Flirty Icebreakers</t>
         </is>
       </c>
     </row>
@@ -355,7 +355,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admit the most childish thing that still genuinely upsets you.</t>
+          <t xml:space="preserve">What's an instant turn-on that has nothing to do with looks?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -365,7 +365,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Confessions</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -377,7 +377,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather always be ten minutes late or twenty minutes early, forever?</t>
+          <t xml:space="preserve">What's the most attractive quality someone can have?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -387,7 +387,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">This or That</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -399,7 +399,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather read minds or be invisible for a day? Justify the chaos.</t>
+          <t xml:space="preserve">Where's your favorite place to be kissed that you'd say out loud?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -409,7 +409,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">This or That</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -421,7 +421,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather lose all your photos or all your texts?</t>
+          <t xml:space="preserve">What's a small thing someone does that drives you a little wild?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -431,7 +431,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">This or That</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -443,7 +443,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather never drink again or never check your phone again? Choose carefully.</t>
+          <t xml:space="preserve">What's the most attractive way someone has ever flirted with you?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -453,7 +453,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">This or That</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiss, marry, avoid: three people the group picks for you.</t>
+          <t xml:space="preserve">Confess the celebrity you'd completely embarrass yourself for.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -475,7 +475,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">This or That</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give {{randomOtherPlayer}} the most convincing compliment you can, no laughing.</t>
+          <t xml:space="preserve">What outfit makes you feel the most irresistible?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -497,7 +497,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your ideal first date in enough detail to make {{randomOtherPlayer}} jealous.</t>
+          <t xml:space="preserve">What's the sexiest non-sexy thing someone can do?</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -531,7 +531,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the first thing you notice about someone across a room?</t>
+          <t xml:space="preserve">Describe your dream first kiss in detail.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell {{randomOtherPlayer}} one thing that would instantly win you over.</t>
+          <t xml:space="preserve">What's your biggest weakness in someone you're attracted to?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -563,7 +563,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's your most attractive quality? Brag, don't be humble.</t>
+          <t xml:space="preserve">Who here would you swipe right on with no hesitation?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Look at {{randomOtherPlayer}} and guess their toxic dating trait.</t>
+          <t xml:space="preserve">What's the flirtiest text you've ever sent sober?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -607,7 +607,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -619,7 +619,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the smoothest thing anyone has ever said to you?</t>
+          <t xml:space="preserve">What's the quickest way to make you catch feelings?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -629,7 +629,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate the group's collective flirting skills and name a clear winner.</t>
+          <t xml:space="preserve">What body part do you notice first? Be honest.</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Light Flirtation</t>
+          <t xml:space="preserve">Turn-Ons &amp; Attraction</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's ever rehearsed a text before sending it, drink.</t>
+          <t xml:space="preserve">Would you rather be irresistibly hot or unbelievably charming?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's stalked an ex's profile this week, drink twice.</t>
+          <t xml:space="preserve">Would you rather kiss the best kisser here or the best looking?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's lied about how much they've had tonight, drink.</t>
+          <t xml:space="preserve">Would you rather always make the first move or always be pursued?</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's the messiest one in their friend group, drink; you know who you are.</t>
+          <t xml:space="preserve">Would you rather date someone way too hot or way too into you?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's ever faked being busy to avoid plans, take a sip.</t>
+          <t xml:space="preserve">Would you rather have your search history or your DMs read aloud?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -761,7 +761,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's cried in the last week, the group drinks for you.</t>
+          <t xml:space="preserve">Kiss, marry, avoid: three people the group picks for you.</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone still a little hung up on someone they shouldn't be, drink.</t>
+          <t xml:space="preserve">Would you rather be caught staring or caught blushing?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's ever been called intimidating, drink and take the compliment.</t>
+          <t xml:space="preserve">Would you rather be someone's fantasy or their favorite mistake?</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Social)</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do your best impression of another player until someone guesses who it is.</t>
+          <t xml:space="preserve">Would you rather get a love letter or a very forward text?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Speak in your most dramatic movie-trailer voice until your next turn; break character and drink.</t>
+          <t xml:space="preserve">Would you rather flirt badly or never flirt at all?</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Sexy This or That</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let the group pick your next social media caption, no editing.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} your best bedroom eyes for 10 seconds without laughing.</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the group the last photo you took, then explain it with no context.</t>
+          <t xml:space="preserve">Whisper something flirty in {{randomOtherPlayer}}'s ear, or drink 2.</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do your most convincing runway walk across the room.</t>
+          <t xml:space="preserve">Compliment {{randomOtherPlayer}}'s best feature while holding eye contact, or drink.</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} give you a nickname for the rest of the night.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} an uninterrupted 15-second compliment about how they look tonight.</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read your last sent text out loud in a seductive whisper.</t>
+          <t xml:space="preserve">Sit close on {{randomOtherPlayer}}'s side for the next round, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone votes: who's most likely to get famous, and for what? Winner gives out 2 drinks.</t>
+          <t xml:space="preserve">Do your slowest, most seductive walk across the room.</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold eye contact with {{randomOtherPlayer}} for 20 seconds; first to laugh drinks.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a 15-second shoulder rub like you mean it.</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compliment everyone in the room in one breath; miss someone and drink twice.</t>
+          <t xml:space="preserve">Look {{randomOtherPlayer}} in the eyes and deliver the smoothest line you've got.</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess which player you'd want beside you in a crisis, and why.</t>
+          <t xml:space="preserve">Make your sexiest face at {{randomOtherPlayer}} and let them rate it, or drink 2.</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do your signature dance move like the whole room is watching, because they are.</t>
+          <t xml:space="preserve">Slow dance with {{randomOtherPlayer}} to whatever plays next.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1091,7 +1091,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Playful Dares</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most irrational fear you have that you know makes no sense?</t>
+          <t xml:space="preserve">Whisper which player here you'd least mind being stuck under the mistletoe with.</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">If you had to delete one app right now, which one would actually hurt?</t>
+          <t xml:space="preserve">Feed {{randomOtherPlayer}} the next sip of your drink.</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1135,7 +1135,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a trend you pretended to understand just to fit in?</t>
+          <t xml:space="preserve">Trace a slow line down {{randomOtherPlayer}}'s arm, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the pettiest thing that instantly makes you judge someone?</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a nickname you'd only use in private.</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your last group-chat drama in exactly one sentence.</t>
+          <t xml:space="preserve">Bite your lip and hold eye contact with {{randomOtherPlayer}} for 10 seconds; first to laugh drinks.</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a compliment you got once that you still think about?</t>
+          <t xml:space="preserve">Read your last text out loud in your most seductive voice.</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the one word your friends would use to describe you behind your back?</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} fix your hair or collar, slowly, or drink 2.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Icebreakers &amp; Wit</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admit the last time you pretended to be busy to get out of something.</t>
+          <t xml:space="preserve">Say the most flirtatious thing you can to {{randomOtherPlayer}} with a straight face.</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Flirty Dares</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most embarrassing thing you've done while completely sober?</t>
+          <t xml:space="preserve">Drink if you've got a crush on someone in this room.</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess a lie you've told to seem cooler than you actually are.</t>
+          <t xml:space="preserve">Drink if you've checked someone out tonight.</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the pettiest revenge you've ever taken?</t>
+          <t xml:space="preserve">Take a sip for every person here you'd consider kissing.</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell the group your most embarrassing autocorrect disaster.</t>
+          <t xml:space="preserve">Drink if you're a shameless flirt once you've had a few.</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's something everyone seems to love that you secretly can't stand?</t>
+          <t xml:space="preserve">Drink if you've re-read a flirty text just to feel something.</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Confessions</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather always say exactly what you're thinking or never speak your mind again?</t>
+          <t xml:space="preserve">Drink if you've ever had a crush on a friend.</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">More This or That</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather be slightly too honest or slightly too fake for a year?</t>
+          <t xml:space="preserve">Drink if you've kissed someone within an hour of meeting them.</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">More This or That</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather relive your most embarrassing moment or your worst-ever haircut?</t>
+          <t xml:space="preserve">Drink if you came out tonight secretly hoping to meet someone.</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">More This or That</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Would you rather have every text you've sent read aloud or every photo shown?</t>
+          <t xml:space="preserve">Drink if you've got a type and everyone already knows it.</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">More This or That</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell {{randomOtherPlayer}} the most attractive thing about their personality.</t>
+          <t xml:space="preserve">Drink if you've ever sent a risky text and instantly regretted it.</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the biggest green flag in someone you're into?</t>
+          <t xml:space="preserve">Anyone who's the flirtiest one in their friend group, drink twice.</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guess {{randomOtherPlayer}}'s love language; they tell you if you nailed it.</t>
+          <t xml:space="preserve">Drink if you've had a dream about someone in this room.</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the fastest way to your heart, in your experience?</t>
+          <t xml:space="preserve">Drink if you'd say yes to a kiss dare right now.</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your ideal partner in three words, then look at who's closest in the room.</t>
+          <t xml:space="preserve">Drink if there's someone here you'd let walk you home.</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Drink If (Flirty)</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a small thing someone can do that you find weirdly attractive?</t>
+          <t xml:space="preserve">Confess the last time someone made you nervous in a good way.</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1597,7 +1597,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Light Flirtation</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's re-read a text after sending it just to check the tone, drink.</t>
+          <t xml:space="preserve">Reveal your most-used pickup line, or drink 2.</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Social)</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's ghosted someone this year, drink twice.</t>
+          <t xml:space="preserve">Describe the best kiss of your life without naming names.</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Social)</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who gives relationship advice they don't actually follow, drink.</t>
+          <t xml:space="preserve">Admit which player here you'd want as your spin-the-bottle partner.</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Social)</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's saved a screenshot to overanalyze later, drink.</t>
+          <t xml:space="preserve">Tell the group your biggest flirting red flag.</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Social)</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1697,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's ever left someone on read on purpose, drink.</t>
+          <t xml:space="preserve">Confess a time you embarrassed yourself over someone hot.</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1707,7 +1707,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Social)</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} choose an accent you have to keep until your next turn; slip and drink.</t>
+          <t xml:space="preserve">Say the most flirtatious thing you can to the person on your left.</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1741,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text the third person in your recent messages a single heart emoji; screenshot the send or drink 2.</t>
+          <t xml:space="preserve">Reveal what someone has to do to instantly win you over.</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do your most convincing fake laugh until someone else laughs for real.</t>
+          <t xml:space="preserve">Rate the room's collective flirting game and crown a winner; they give out 2 drinks.</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give the group your honest first impression of {{randomOtherPlayer}}.</t>
+          <t xml:space="preserve">Tell {{randomOtherPlayer}} one thing they do that's lowkey attractive.</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1807,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let the group ask you one embarrassing question; answer honestly or drink 2.</t>
+          <t xml:space="preserve">Confess who gave you your most memorable first-kiss story.</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1817,7 +1817,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the group your screen time for today, no hiding, or drink 2.</t>
+          <t xml:space="preserve">Reveal how you act when you're into someone: obvious, sneaky, or clueless?</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Playful Dares</t>
+          <t xml:space="preserve">Tension &amp; Reveals</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe the most awkward hookup you've ever had; spare no cringe.</t>
+          <t xml:space="preserve">What's the craziest place you've ever hooked up?</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the worst place you've ever been caught making out?</t>
+          <t xml:space="preserve">Describe your wildest hookup without naming names.</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1895,7 +1895,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the wildest thing you've done to impress someone you wanted.</t>
+          <t xml:space="preserve">What's the dirtiest text you've ever sent? Read it or drink 3.</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell the story of your worst date, the one that became a group legend.</t>
+          <t xml:space="preserve">Confess your go-to fantasy, at least the tame version of it.</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the boldest way you've ever shot your shot?</t>
+          <t xml:space="preserve">What's the most trouble you've gotten into over hooking up with someone?</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the most trouble a crush has ever gotten you into.</t>
+          <t xml:space="preserve">What's your body count range? Give us hot, cold, or 'no comment' and drink 2.</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1971,7 +1971,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read the dirtiest text you've ever sent, verbatim, or drink 3.</t>
+          <t xml:space="preserve">Confess the hottest thing someone has ever said to you in bed.</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -1993,7 +1993,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the closest you've come to getting caught doing something you shouldn't?</t>
+          <t xml:space="preserve">What's the closest you've come to getting caught in the act?</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess a fantasy that has nothing to do with anyone in this room. Probably.</t>
+          <t xml:space="preserve">Describe your type in bed in one sentence.</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most reckless thing you've done for a good story?</t>
+          <t xml:space="preserve">What's the boldest thing you've done to seduce someone?</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2071,7 +2071,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe the best kiss of your life without naming any names.</t>
+          <t xml:space="preserve">Confess a hookup you'd absolutely repeat tonight if you could.</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the most delusional situationship you convinced yourself was real.</t>
+          <t xml:space="preserve">What's the most spontaneous sex you've ever had?</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spicy Confessions &amp; Stories</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's your favorite feature on {{randomOtherPlayer}}? Be specific.</t>
+          <t xml:space="preserve">Reveal the wildest place you'd be down to get frisky.</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2125,7 +2125,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2137,7 +2137,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Where do you love being kissed that isn't your mouth?</t>
+          <t xml:space="preserve">What's your favorite thing to do to someone you're into?</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2159,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's an instant turn-on for you that has nothing to do with looks?</t>
+          <t xml:space="preserve">Confess the last thing you did that would make your mother faint.</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2181,7 +2181,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">If you had to make out with one person here, who's the least bad option?</t>
+          <t xml:space="preserve">What's the sexiest dream you've had recently?</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2203,7 +2203,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's your type, and who in this room is dangerously close to it?</t>
+          <t xml:space="preserve">Describe exactly how you like to be kissed.</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most attractive thing someone can do while fully clothed?</t>
+          <t xml:space="preserve">What's a turn-on you're a little embarrassed about?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who in this room gives the most trouble energy, and do you mean it as a compliment?</t>
+          <t xml:space="preserve">What's the hottest hookup story your friends know you for?</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2269,7 +2269,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">What does someone have to do to make you catch feelings against your will?</t>
+          <t xml:space="preserve">What's your biggest 'I shouldn't, but I would' about someone here?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Point to who you'd least want to see your search history; they drink 2.</t>
+          <t xml:space="preserve">Are you louder or quieter than people would expect? Confess or drink 2.</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">How fast has someone ever gone from a stranger to exactly your type?</t>
+          <t xml:space="preserve">What's the most daring thing you've done somewhere semi-public?</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the longest dry spell you'll admit to? Drink for every month you'd rather not say.</t>
+          <t xml:space="preserve">Reveal your dirtiest guilty-pleasure fantasy scenario.</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Questions</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever fantasized about someone in this room.</t>
+          <t xml:space="preserve">What's the fastest you've ever gone from flirting to a lot more?</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Take a drink for every person here you've thought about more than once.</t>
+          <t xml:space="preserve">Confess the wildest thing you've said yes to in the heat of the moment.</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Confessions</t>
         </is>
       </c>
     </row>
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever sent a text you'd be mortified to have read aloud.</t>
+          <t xml:space="preserve">What's your favorite part of {{randomOtherPlayer}}'s body? Be specific.</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've hooked up with someone and never told your friends.</t>
+          <t xml:space="preserve">Where do you most love being touched?</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever faked it convincingly enough to get an encore.</t>
+          <t xml:space="preserve">If you had to hook up with one person here, who and why?</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2467,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if your body count is higher than your closest friend would guess.</t>
+          <t xml:space="preserve">What's the sexiest thing someone can do with their hands?</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever hooked up with a coworker, a roommate, or a regret.</t>
+          <t xml:space="preserve">Dominant or submissive? Prove it or drink 2.</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2511,7 +2511,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've sent a spicy photo in the last month.</t>
+          <t xml:space="preserve">What's your ideal way to be woken up by someone?</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Take a sip for every dating app on your phone right now.</t>
+          <t xml:space="preserve">Who in this room gives the best 'take me home' energy?</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever gone home with someone you met that same night.</t>
+          <t xml:space="preserve">What's an instant turn-on that gets you every single time?</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've hooked up somewhere you could easily have been caught.</t>
+          <t xml:space="preserve">What would you do to {{randomOtherPlayer}} if the lights went out for a minute?</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever flirted your way out of a ticket, a bill, or trouble.</t>
+          <t xml:space="preserve">What's your dirtiest thought right now? Say it or drink 3.</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if there's someone here you'd say yes to right now.</t>
+          <t xml:space="preserve">Where's the most adventurous place you'd want to try something?</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2631,7 +2631,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2643,7 +2643,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's been the reason a couple broke up, drink; no elaboration required.</t>
+          <t xml:space="preserve">What's the quickest way to turn you on without touching you?</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who owns something they'd hide before a parent visited, drink twice.</t>
+          <t xml:space="preserve">Who here would you pick for a no-strings night? Point or drink 3.</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink If (Sexual History)</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone vote: who here is secretly the wildest in private? They drink 2.</t>
+          <t xml:space="preserve">What's your favorite position, in as few words as possible?</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vote for who gives the best hugs; the winner earns a demonstration or gives out 2 drinks.</t>
+          <t xml:space="preserve">What's a kink you're at least a little curious about?</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2719,7 +2719,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who's most likely to have a spicy secret account? They drink 3, or prove you wrong.</t>
+          <t xml:space="preserve">What sound or word instantly gets you going?</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2753,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone point at once: who's the best kisser in the room? The winner gives out 5.</t>
+          <t xml:space="preserve">If {{randomOtherPlayer}} made a move right now, what's your honest reaction?</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2775,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vote for who's most likely to break a heart this year; they drink 2.</t>
+          <t xml:space="preserve">What's the hottest thing about the person to your left?</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2797,7 +2797,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone votes for who they'd trust with their phone unlocked; least trusted drinks 4.</t>
+          <t xml:space="preserve">How do you like it: slow and teasing, or fast and reckless?</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2819,7 +2819,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who here could talk anyone into anything? They give out 3 drinks.</t>
+          <t xml:space="preserve">What's the most attractive thing someone can whisper to you?</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vote: who's most likely to text an ex tonight? They hand over their phone or drink 3.</t>
+          <t xml:space="preserve">Who in this room is secretly the freakiest? They drink 3.</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -2851,7 +2851,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2863,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone votes: who's the biggest flirt at this table? They give out 3 drinks.</t>
+          <t xml:space="preserve">What's your biggest green light that someone's about to get lucky?</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Dirty Questions</t>
         </is>
       </c>
     </row>
@@ -2885,7 +2885,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Whisper something you find attractive about {{randomOtherPlayer}} in their ear, or drink 1.</t>
+          <t xml:space="preserve">Drink if you've ever fantasized about someone in this room.</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give {{randomOtherPlayer}} a 20-second shoulder massage like you mean it.</t>
+          <t xml:space="preserve">Take a drink for every person here you've thought about that way.</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trace a slow line from {{randomOtherPlayer}}'s wrist to their elbow, or take 1 drinks.</t>
+          <t xml:space="preserve">Drink if you've hooked up somewhere you could've been caught.</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold {{randomOtherPlayer}}'s gaze and describe how you'd greet them after a year apart.</t>
+          <t xml:space="preserve">Drink if you've ever faked it convincingly.</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Feed {{randomOtherPlayer}} the next sip of your drink.</t>
+          <t xml:space="preserve">Drink if you've sent a nude in the last month.</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -2995,7 +2995,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} whisper something scandalous in your ear; keep a straight face or drink.</t>
+          <t xml:space="preserve">Drink if you've had a one-night stand.</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Slow dance with {{randomOtherPlayer}} to whatever plays next, no matter the tempo.</t>
+          <t xml:space="preserve">Drink if you've hooked up with a coworker.</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give {{randomOtherPlayer}} your best bedroom eyes for 10 seconds without laughing.</t>
+          <t xml:space="preserve">Drink if you've had sex somewhere other than a bed.</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sit on {{randomOtherPlayer}}'s lap until your next turn, or take 2 drinks.</t>
+          <t xml:space="preserve">Drink if your body count is higher than people would guess.</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Compliment {{randomOtherPlayer}}'s best physical feature while holding eye contact, or drink 1.</t>
+          <t xml:space="preserve">Drink if you've hooked up with an ex you swore you were done with.</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} write a word on your arm with a fingertip; guess it or drink.</t>
+          <t xml:space="preserve">Drink if you've had a friends-with-benefits situation.</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -3115,7 +3115,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do your best impression of {{randomOtherPlayer}} flirting; they rate it or drink 1.</t>
+          <t xml:space="preserve">Drink if you've ever sexted at work.</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sensual Dares (Light)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal your go-to pickup line to give out 3 drinks, or drink 1 to keep it secret.</t>
+          <t xml:space="preserve">Drink if you've gone home with someone the night you met them.</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Say your body count out loud to give out 3 drinks, or drink 2 to keep the mystery.</t>
+          <t xml:space="preserve">Drink if you own a toy within reach of your bed.</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the group the last spicy text you sent to give out 3 drinks.</t>
+          <t xml:space="preserve">Drink if you've ever moaned the wrong name.</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name the ick that ends things for you instantly; anyone guilty of it drinks.</t>
+          <t xml:space="preserve">Drink if you've had a crush on someone completely off-limits.</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -3225,7 +3225,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your ideal night in with someone in enough detail to give out 3 drinks.</t>
+          <t xml:space="preserve">Drink if you've got a hookup you can't tell your friends about.</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3247,7 +3247,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3259,7 +3259,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal the wildest place you'd be willing to get frisky to give out 3 drinks.</t>
+          <t xml:space="preserve">Drink if you've hooked up with someone in this friend group.</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admit which player you'd swipe right on to give out 3 drinks, or drink 1.</t>
+          <t xml:space="preserve">Drink if you've ever recorded, or been recorded.</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3303,7 +3303,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess a crush you had that would genuinely surprise everyone here, or drink 2.</t>
+          <t xml:space="preserve">Drink if you've had sex in a car.</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveals (Incentivized)</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Text your most recent crush a single 👀 and show the group the send, or drink 3.</t>
+          <t xml:space="preserve">Drink if you've ever hooked up on a first date.</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the group your most recent selfie, the one you didn't post, or drink 2.</t>
+          <t xml:space="preserve">Drink if you've done something tonight you'd deny tomorrow.</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read your boldest DM out loud, or drink 3.</t>
+          <t xml:space="preserve">Drink if you've had a purely physical thing with someone.</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let the group ask you one yes-or-no question about your love life; answer or drink 2.</t>
+          <t xml:space="preserve">Anyone who's had a work crush turn into more, drink twice.</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trade phones with {{randomOtherPlayer}} for one round; no deleting.</t>
+          <t xml:space="preserve">Drink if there's someone here you'd say yes to right now.</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3423,7 +3423,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} post a one-word story to your close friends, or drink 3.</t>
+          <t xml:space="preserve">Drink if you've hooked up with someone twice in one night.</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phone &amp; Reveal Stunts</t>
+          <t xml:space="preserve">Drink If (Sexual History)</t>
         </is>
       </c>
     </row>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone showing skin below the collarbone right now, drink twice.</t>
+          <t xml:space="preserve">Everyone vote: who's the best kisser in the room? Winner gives out 3.</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t xml:space="preserve">The last person here to hook up with someone, drink 2; welcome back.</t>
+          <t xml:space="preserve">Who here is most likely to be a freak behind closed doors? They drink 3.</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone single by choice, drink. Everyone single by circumstance, drink twice.</t>
+          <t xml:space="preserve">Vote for who has the best body in the room; they give out 3 drinks.</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3523,7 +3523,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's ever dated someone in this room, or wanted to, drink.</t>
+          <t xml:space="preserve">Who's most likely to have a secret spicy account? They drink 3, or prove you wrong.</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t xml:space="preserve">The most recently heartbroken person here finishes their drink; the group toasts you.</t>
+          <t xml:space="preserve">Everyone point: who would you most want a lap dance from? They give out 3.</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -3555,7 +3555,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3567,7 +3567,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone born under a fire sign, drink 2 and act surprised.</t>
+          <t xml:space="preserve">Who gives the most 'dangerous to be alone with' energy? They drink 2.</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -3577,7 +3577,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3589,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who thinks they're the best-looking person in the room, drink; bold move.</t>
+          <t xml:space="preserve">Vote for who's most likely to make the first move tonight; they drink 2.</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's ever been called a heartbreaker, give out 2 drinks.</t>
+          <t xml:space="preserve">Who here has the best lips? Everyone who agrees drinks.</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -3621,7 +3621,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Take a drink for every year since your last relationship; round up.</t>
+          <t xml:space="preserve">Who's the biggest tease in the room? They give out 3 drinks.</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3643,7 +3643,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3655,7 +3655,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone wearing black tonight, drink; you know exactly what you're doing.</t>
+          <t xml:space="preserve">Vote for who'd win a make-out competition; they pick their partner or drink 3.</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3677,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone not wearing socks right now, take a drink.</t>
+          <t xml:space="preserve">Who's most likely to send a 2am 'you up?' text? They drink 2.</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -3687,7 +3687,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t xml:space="preserve">The person who's checked their phone most this round drinks twice.</t>
+          <t xml:space="preserve">Who has the best ass in the room? Winner gives out 3 drinks.</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Social Drink Commands</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3721,7 +3721,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reenact the face you make when a text from a crush lights up your phone.</t>
+          <t xml:space="preserve">Vote for the horniest person here; they finish their drink.</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Sexual Voting &amp; Group Heat</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Whisper the number of people you've kissed to {{randomOtherPlayer}}; they decide if the group finds out.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a lap dance for 15 seconds, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3765,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rank the room by who you'd want stranded on an island with; most romantic reasons win a drink to give out.</t>
+          <t xml:space="preserve">Sit on {{randomOtherPlayer}}'s lap for the next two rounds.</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Admit the pettiest thing you've done after a breakup, or drink 2.</t>
+          <t xml:space="preserve">Whisper the dirtiest thing you're comfortable saying into {{randomOtherPlayer}}'s ear, or drink 3.</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3797,7 +3797,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3809,7 +3809,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} choose one word you have to work into conversation until your next turn; fail and drink.</t>
+          <t xml:space="preserve">Grind on {{randomOtherPlayer}} for 10 seconds, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -3819,7 +3819,7 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your worst kiss ever without naming who it was with.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a slow massage from shoulders to lower back, or drink 3.</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone vote for the biggest tease in the room; they give out 3 drinks.</t>
+          <t xml:space="preserve">Kiss {{randomOtherPlayer}} on the cheek, neck, or lips, their choice, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the last thing that made you blush, or drink 2.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} whisper where they'd kiss you first, or drink 2.</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Look at {{randomOtherPlayer}} and finish this sentence out loud: 'If we were alone right now...'</t>
+          <t xml:space="preserve">Trace your fingers slowly up {{randomOtherPlayer}}'s arm and neck, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give {{randomOtherPlayer}} a genuine, uninterrupted 15-second compliment; no jokes allowed.</t>
+          <t xml:space="preserve">Straddle a chair and give {{randomOtherPlayer}} your best tease, or drink 3.</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3929,7 +3929,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal the most attractive thing about the last person you dated, or drink 1.</t>
+          <t xml:space="preserve">Slow dance with {{randomOtherPlayer}} close enough to feel their heartbeat, or drink 2.</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3963,7 +3963,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's ever kept a hookup a secret from this exact group, drink.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} run their hands through your hair for 15 seconds, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flirty Challenges</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the most inappropriate time you've caught yourself flirting.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a soft neck kiss for 5 seconds, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4007,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the wildest thing you've done just because someone dared you?</t>
+          <t xml:space="preserve">Sit back-to-front on {{randomOtherPlayer}}'s lap for one round, or drink 3.</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -4017,7 +4017,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe your worst 'what was I thinking' hookup, no names.</t>
+          <t xml:space="preserve">Do a 15-second sexy dance for the group, or finish your drink.</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the pettiest reason you've ever swiped left on someone?</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} feed you a shot from their hand, or drink 2.</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4073,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the last time you flirted purely for the attention.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} place your hands wherever they want them for 10 seconds, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most embarrassing thing you've done to keep someone interested?</t>
+          <t xml:space="preserve">Press up against {{randomOtherPlayer}} and slow dance for a full song, or drink 3.</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell the group about the one that got away, or drink 2.</t>
+          <t xml:space="preserve">Whisper a rating of how good you think {{randomOtherPlayer}} is in bed, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the closest you've ever come to a public scandal?</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} undo one of your buttons, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confess the boldest lie you've told to get out of a bad date.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} your best over-the-clothes tease for 10 seconds, or drink 3.</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Describe the moment you realized you were way too into someone.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} pick a spot above the waist to kiss, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's a hookup story your friends still won't let you live down?</t>
+          <t xml:space="preserve">Sit thigh-to-thigh with {{randomOtherPlayer}} and describe your ideal night together, or drink 2.</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -4215,7 +4215,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most trouble a text has ever gotten you into?</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} a 10-second lap dance facing them, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4237,7 +4237,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Spicy Confessions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who in this room would you most want to be stranded with overnight?</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} trace a word on your lower back; guess it or drink 2.</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4271,7 +4271,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the most attractive thing {{randomOtherPlayer}} is wearing right now?</t>
+          <t xml:space="preserve">Demonstrate your best slow grind on the nearest chair, or finish your drink.</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Hands-On Dares</t>
         </is>
       </c>
     </row>
@@ -4293,7 +4293,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t xml:space="preserve">If you had to kiss someone here to save your life, who and where?</t>
+          <t xml:space="preserve">Show the group the last spicy text you sent, or drink 3.</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4315,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's your most shameless move when you're actually interested in someone?</t>
+          <t xml:space="preserve">Text your latest crush something flirty right now, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4337,7 +4337,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who here has the most dangerous smile? They give out 2 drinks.</t>
+          <t xml:space="preserve">Read your dirtiest saved message out loud, or finish your drink.</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4347,7 +4347,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's the quickest someone has ever turned you on without touching you?</t>
+          <t xml:space="preserve">Reveal the name of the last person you sexted, or drink 3.</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4369,7 +4369,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t xml:space="preserve">If {{randomOtherPlayer}} asked you out right now, what's your honest answer?</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} send one flirty emoji to your most recent match, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who in this room is most your type physically? Say it or drink 2.</t>
+          <t xml:space="preserve">Reveal how many people you're texting right now, or drink 2.</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4425,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t xml:space="preserve">What's an outfit that instantly gets your attention on someone?</t>
+          <t xml:space="preserve">Show your most recent selfie you didn't post, or drink 2.</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t xml:space="preserve">What would your perfect night alone with someone you wanted actually look like?</t>
+          <t xml:space="preserve">Read your last DM to a crush in your sexiest voice, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rate how good a kisser you think you are, then find someone here to confirm it.</t>
+          <t xml:space="preserve">Let the group write a flirty text you have to actually send, or finish your drink.</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -4479,7 +4479,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who here would you trust to pick your outfit for a first date? They give out 2 drinks.</t>
+          <t xml:space="preserve">Text 'thinking about you' to someone and screenshot the reply, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Flirty Questions</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever had a crush on a friend's ex.</t>
+          <t xml:space="preserve">Reveal the wildest thing in your search history, or drink 3.</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Sexting &amp; Phone</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever kissed someone within an hour of meeting them.</t>
+          <t xml:space="preserve">Say your body count out loud to give out 3 drinks, or drink 2 to keep it secret.</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever pretended to like someone just for the attention.</t>
+          <t xml:space="preserve">Reveal your kinkiest turn-on to give out 3 drinks.</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -4567,7 +4567,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've been caught checking someone out tonight.</t>
+          <t xml:space="preserve">Describe your dirtiest fantasy to give out 3 drinks, or drink 2.</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever left a party with someone you'd just met.</t>
+          <t xml:space="preserve">Admit which player you'd hook up with to give out 3 drinks, or drink 3.</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've had a hookup you'd repeat but would never admit to.</t>
+          <t xml:space="preserve">Reveal the weirdest place you've had sex to give out 3 drinks.</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4645,7 +4645,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever saved someone's number under a fake name.</t>
+          <t xml:space="preserve">Confess your loudest moment in bed to give out 3 drinks.</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4667,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Take a sip for every person here you've considered as more than a friend.</t>
+          <t xml:space="preserve">Name your ultimate celebrity hall pass and what you'd do, to give out 2 drinks.</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've ever sent a risky text and immediately regretted it.</t>
+          <t xml:space="preserve">Describe your ideal one-night stand to give out 3 drinks.</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -4699,7 +4699,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've shot your shot at someone way out of your league.</t>
+          <t xml:space="preserve">Admit a fantasy involving someone in this room to give out 3 drinks, or drink 3.</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's ever had a serious work crush, drink twice.</t>
+          <t xml:space="preserve">Say the filthiest thing you're willing to; everyone who blushes drinks.</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -4743,7 +4743,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drink if you've re-downloaded a dating app out of pure boredom.</t>
+          <t xml:space="preserve">Reveal your hard yes and hard no in bed to give out 3 drinks.</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Drink If (Sexual History)</t>
+          <t xml:space="preserve">Reveals (Incentivized)</t>
         </is>
       </c>
     </row>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone vote: who's most likely to say yes to a spontaneous adventure? They give out 2 drinks.</t>
+          <t xml:space="preserve">Undo one button or roll up one sleeve; the group decides which, or drink 2.</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -4787,7 +4787,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who here has the best trouble energy? They drink 2.</t>
+          <t xml:space="preserve">Describe what you're wearing underneath, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4821,7 +4821,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vote for who'd last longest on a dating show; the winner gives out 3 drinks.</t>
+          <t xml:space="preserve">Everyone show a little more skin than you were, or drink.</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4843,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who in this room is the biggest secret romantic? They drink 2.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} guess your most sensitive spot; nod or drink 2.</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -4853,7 +4853,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4865,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone point at once: who's most likely to fall in love this year? They drink 2.</t>
+          <t xml:space="preserve">Take off one accessory as seductively as you can, or drink 2.</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4887,7 +4887,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who here would be the most dangerous to share a hotel room with? They give out 3 drinks.</t>
+          <t xml:space="preserve">Let the group vote on one item of yours to lose for the round, or take 3 drinks.</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4909,7 +4909,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone vote: whose DMs are the most chaotic? They hand over their phone or drink 3.</t>
+          <t xml:space="preserve">Describe the last time someone left you breathless, or drink 2.</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -4919,7 +4919,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who's most likely to make the first move tonight? They drink 2.</t>
+          <t xml:space="preserve">Give {{randomOtherPlayer}} your best 'come here' look, or drink 2.</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Voting &amp; Group Heat</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rest your head on {{randomOtherPlayer}}'s shoulder for the next two rounds.</t>
+          <t xml:space="preserve">Whisper your safe-for-now fantasy to {{randomOtherPlayer}}, or take 2 drinks.</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -4963,7 +4963,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Give {{randomOtherPlayer}} a compliment so smooth the whole room groans, or drink 2.</t>
+          <t xml:space="preserve">Let {{randomOtherPlayer}} choose: kiss their cheek or lose a layer.</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -4985,7 +4985,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -4997,7 +4997,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hold hands with {{randomOtherPlayer}} until your next turn; let go early and drink.</t>
+          <t xml:space="preserve">Tell {{randomOtherPlayer}} exactly how you'd start a night alone with them, or drink 3.</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Look {{randomOtherPlayer}} dead in the eyes and say something you'd usually only dare to text.</t>
+          <t xml:space="preserve">Do your most convincing moan; the least convincing player drinks.</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -5029,7 +5029,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Body &amp; Tension</t>
         </is>
       </c>
     </row>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Whisper your favorite thing about tonight into {{randomOtherPlayer}}'s ear.</t>
+          <t xml:space="preserve">Everyone not wearing underwear, drink twice.</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5063,7 +5063,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} slowly fix your hair or collar, or take 2 drinks.</t>
+          <t xml:space="preserve">Anyone showing a little cleavage or chest, drink.</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5085,7 +5085,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tell {{randomOtherPlayer}} exactly how you'd plan a date to impress them.</t>
+          <t xml:space="preserve">Everyone who's hooked up with someone in this room, drink.</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trace the outline of {{randomOtherPlayer}}'s hand with your finger while holding eye contact.</t>
+          <t xml:space="preserve">Anyone who's thought about a hookup tonight, drink.</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} pick a pet name to call you for the rest of the game.</t>
+          <t xml:space="preserve">The horniest person here, be honest, finishes their drink.</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -5139,7 +5139,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5151,7 +5151,7 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Slow dance with {{randomOtherPlayer}} close enough to whisper, or drink 2.</t>
+          <t xml:space="preserve">Everyone who's down to leave with someone tonight, take a sip; no judgment.</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Sensual Dares (Light)</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the group the last search you'd be a little embarrassed by, or drink 3.</t>
+          <t xml:space="preserve">Anyone who's had sex today, drink 3, lucky you.</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -5183,7 +5183,7 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5195,7 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read your last outgoing text in the voice of someone seducing a stranger.</t>
+          <t xml:space="preserve">Everyone who calls themselves a good kisser, prove it or drink 2.</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5217,7 +5217,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal the pet name saved for your most recent crush, or drink 2.</t>
+          <t xml:space="preserve">The last person here to hook up, drink 3.</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -5227,7 +5227,7 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Show the last person you texted 'goodnight', or drink 3.</t>
+          <t xml:space="preserve">Anyone with a toy at home, drink twice.</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -5249,7 +5249,7 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Let {{randomOtherPlayer}} scroll to your oldest saved photo and react to it.</t>
+          <t xml:space="preserve">Everyone who's ever hooked up with a friend, drink.</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Read the first line of your last flirty conversation out loud, or drink 3.</t>
+          <t xml:space="preserve">The person most likely to leave with someone tonight drinks 2 and takes a bow.</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5293,7 +5293,7 @@
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5305,7 +5305,7 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Reveal how many unread dating-app messages you have right now, or drink 2.</t>
+          <t xml:space="preserve">Anyone who's ever had a hookup in this room's company, drink.</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hand your phone to {{randomOtherPlayer}} and let them send one emoji to anyone, or drink 3.</t>
+          <t xml:space="preserve">Everyone who's flirted with someone here tonight, drink.</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Reveals &amp; Phone</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone wearing something they'd happily take off if it got warmer, drink.</t>
+          <t xml:space="preserve">Anyone who's not wearing a bra right now, drink twice.</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5371,7 +5371,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t xml:space="preserve">The best-dressed person here gives out 2 drinks; everyone else votes on who.</t>
+          <t xml:space="preserve">Everyone who's had a threesome fantasy about anyone here, drink.</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5393,7 +5393,7 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's thought about someone in this room in a not-so-friendly way, drink.</t>
+          <t xml:space="preserve">The person who's checked someone out the most tonight drinks 2.</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who came out tonight secretly hoping something might happen, drink twice.</t>
+          <t xml:space="preserve">Anyone who'd fail a lie detector about their body count, drink.</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5437,7 +5437,7 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anyone who's flirted with someone in this room before tonight, drink.</t>
+          <t xml:space="preserve">Everyone who's ever hooked up to get over someone, drink.</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -5447,7 +5447,7 @@
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5459,7 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Everyone who's ever caught feelings faster than they'd admit, drink.</t>
+          <t xml:space="preserve">The best kisser here, by group vote, gives out 3 drinks.</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t xml:space="preserve">More Social Commands</t>
+          <t xml:space="preserve">Sexual Drink Commands</t>
         </is>
       </c>
     </row>

</xml_diff>